<commit_message>
Cotação 05/10: pedido OL Procter (campanha até 16/10) para 60 dias
ol_campanha.py lê o PDF do Painel O.L, calcula a quantidade para 60 dias
de estoque (2 × demanda mensal − estoque) na embalagem da oferta e respeita
o teto do histórico. Itens comprados na campanha saem dos pedidos de
distribuidor (Xarope 44E saiu do pedido SB Log).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BYY9KXCh6eZkQnrYXQ3GHn
</commit_message>
<xml_diff>
--- a/cotacoes/2026-10-05/pedidos/distribuidores/PEDIDO_SBLOG_05-10-2026.xlsx
+++ b/cotacoes/2026-10-05/pedidos/distribuidores/PEDIDO_SBLOG_05-10-2026.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -486,7 +486,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Drogarias Rocha • cotação 05-10-2026 • 2 itens</t>
+          <t>Drogarias Rocha • cotação 05-10-2026 • 1 itens</t>
         </is>
       </c>
     </row>
@@ -567,42 +567,13 @@
       <c r="I5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n">
-        <v>65101</v>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>7590002023228</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>XAROPE 44 E 1,30+13,30MG/ML XPE FR 120ML</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="6" t="n">
-        <v>30.04</v>
-      </c>
-      <c r="G6" s="6" t="n">
-        <v>690.92</v>
-      </c>
-      <c r="H6" s="6" t="n">
-        <v>30.73</v>
-      </c>
-      <c r="I6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="G7" s="8">
-        <f>SUM(G5:G6)</f>
+      <c r="G6" s="8">
+        <f>SUM(G5:G5)</f>
         <v/>
       </c>
     </row>

</xml_diff>